<commit_message>
debuggin for varaint-create button in trouser shopsy
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/data inputs/common/Variants-excel.xlsx
+++ b/Full-LC-AUTO/data inputs/common/Variants-excel.xlsx
@@ -1,27 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESHAAN\HAKUR\work--fk-tools\Full-LC-AUTO\data inputs\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{835BAF0D-AB13-4D27-8069-6772164C369A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="20730" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="Jeans Variant Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="Jeans Variant Guide" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
   <si>
     <t>kind</t>
   </si>
@@ -92,8 +86,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -425,14 +419,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -455,7 +449,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -478,7 +472,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -501,7 +495,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -524,7 +518,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -544,7 +538,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -564,15 +558,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>21</v>
       </c>
       <c r="B7">
         <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>7</v>
       </c>
       <c r="D7">
         <v>30</v>
@@ -587,11 +578,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -599,7 +590,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -607,7 +598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -615,7 +606,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -623,7 +614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -631,7 +622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -639,7 +630,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
IMAGE-CHECK POLISH in LC
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/data inputs/common/Variants-excel.xlsx
+++ b/Full-LC-AUTO/data inputs/common/Variants-excel.xlsx
@@ -1,27 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESHAAN\HAKUR\work--fk-tools\Full-LC-AUTO\data inputs\common\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0F5B3513E9574E14FEC18C6D6074A9F54027CA0C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Jeans Variant Inputs" sheetId="1" r:id="rId1"/>
-    <sheet name="Jeans Variant Guide" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="Jeans Variant Inputs" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Jeans Variant Guide" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
   <si>
     <t>kind</t>
   </si>
@@ -47,24 +38,9 @@
     <t>Beige</t>
   </si>
   <si>
-    <t>28</t>
-  </si>
-  <si>
     <t>Number</t>
   </si>
   <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
     <t>Ice</t>
   </si>
   <si>
@@ -93,6 +69,9 @@
   </si>
   <si>
     <t>S</t>
+  </si>
+  <si>
+    <t>Track Pant</t>
   </si>
   <si>
     <t>column</t>
@@ -119,14 +98,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -156,7 +135,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -489,16 +468,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="34.796875" customWidth="1"/>
-    <col min="2" max="7" width="41.5" customWidth="1"/>
-    <col min="8" max="26" width="16.69921875" customWidth="1"/>
+    <col min="1" max="1" width="34.857142857142854" customWidth="1"/>
+    <col min="2" max="7" width="41.57142857142857" customWidth="1"/>
+    <col min="8" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -521,229 +500,245 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2">
+        <v>26</v>
+      </c>
+      <c r="E2">
+        <v>30</v>
+      </c>
+      <c r="F2">
+        <v>32</v>
+      </c>
+      <c r="G2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B3">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3">
+        <v>26</v>
+      </c>
+      <c r="E3">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>32</v>
+      </c>
+      <c r="G3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B4">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>26</v>
+      </c>
+      <c r="E4">
+        <v>30</v>
+      </c>
+      <c r="F4">
+        <v>32</v>
+      </c>
+      <c r="G4">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="B5">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>26</v>
+      </c>
+      <c r="E5">
+        <v>30</v>
+      </c>
+      <c r="F5">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="B6">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>26</v>
+      </c>
+      <c r="E6">
+        <v>30</v>
+      </c>
+      <c r="F6">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B7">
+        <v>28</v>
+      </c>
+      <c r="D7">
+        <v>30</v>
+      </c>
+      <c r="E7">
+        <v>32</v>
+      </c>
+      <c r="F7">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C8" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="D8" t="s">
         <v>16</v>
       </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="E8" t="s">
         <v>17</v>
       </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="F8" t="s">
         <v>18</v>
       </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" t="s">
         <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:G8" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="41.5" customWidth="1"/>
-    <col min="3" max="26" width="16.69921875" customWidth="1"/>
+    <col min="1" max="2" width="41.57142857142857" customWidth="1"/>
+    <col min="3" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:B7" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>